<commit_message>
Add official 31-province data calibration package
</commit_message>
<xml_diff>
--- a/data/public/public_data_catalog.xlsx
+++ b/data/public/public_data_catalog.xlsx
@@ -2,15 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Bank FAO" sheetId="1" r:id="R73f49e8ea1824b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA Annual" sheetId="2" r:id="R31501a7175cc4065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA 2024 Detail" sheetId="3" r:id="Re7da372da256433e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment 2024" sheetId="4" r:id="Rc7668d192654450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latest Official" sheetId="5" r:id="Re9f40b0d25984bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Catalog" sheetId="6" r:id="R8194c3b76d0a48dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="7" r:id="R4551b3800cbe43ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="8" r:id="R9af9c44bc0574012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QC Checks" sheetId="9" r:id="R36b18f2915234f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Bank FAO" sheetId="1" r:id="R08156eea567241b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA Annual" sheetId="2" r:id="Rb20ef625f1624b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA 2024 Detail" sheetId="3" r:id="R6684363ea5aa4080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment 2024" sheetId="4" r:id="R1b650a986aa34698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latest Official" sheetId="5" r:id="R60adbca9c8474aec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NBS 2024 Provinces" sheetId="6" r:id="Re6a9d7edc8974d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NBS Field Dictionary" sheetId="7" r:id="R5b5a5e0e5a784bfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NBS National QC" sheetId="8" r:id="Rbd94b78c41e5443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Catalog" sheetId="9" r:id="R03089fa636a44783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="10" r:id="R6ddad8d6835e4691"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="11" r:id="R44129eb1a8ec47fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QC Checks" sheetId="12" r:id="R395f6b283a894092"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -138,6 +141,18 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -1683,6 +1698,720 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="96" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>Public fishery data package</x:v>
+      </x:c>
+      <x:c r="B1" s="28" t="str">
+        <x:v>Review workbook for the GitHub reproduction repository</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>Retrieved</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>2026-07-23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>Data label</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>经过处理的数据（公开来源） / processed data from public sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>World Bank / FAO</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Three China national production indicators, 2014-2023, CC BY 4.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>Ministry annual data</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>Accessible official HTML communiqués for 2015, 2016 and 2019-2024</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>MOA 2024 detail</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>99 records: economy, species/water-body production, area, fleet, population, processing, trade and disasters</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>Fishery environment</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>12 records: monitoring network and reported exceedance-area change magnitudes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>Latest official</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>2025 national total/aquaculture/capture and Zhejiang total/marine/freshwater production</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>NBS 2024 provinces</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>31 rows from six official yearbook tables: production, population, income, wastewater, freight and e-commerce</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>NBS evidence split</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>Official observations are separate from all later processed/calibrated model fields</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>NBS national QC</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Printed national totals and documented scope/rounding differences used for reconciliation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>Reported vs normalized</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Reported value/unit are retained; normalized value = reported value × normalization multiplier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>Source integrity</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Detailed rows contain the SHA-256 of the official HTML used by the parser</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>Province-level data</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>A0407 returned HTTP 403; direct official yearbook Table 12-15 was used instead</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="32" t="str">
+        <x:v>Important</x:v>
+      </x:c>
+      <x:c r="B15" s="32" t="str">
+        <x:v>World Bank/FAO, Ministry and NBS totals can use different definitions; do not merge without checking scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>Missing values</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>not_found means the field was not located in that official HTML page; no interpolation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>https://github.com/niqundaye/Frontiers-in-Marine-Science</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>Applies to</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>Audit rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>all data sheets</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>Reference year of the statistic</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>Integer year</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>section</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>MOA 2024 Detail</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>Communique topic group</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="str">
+        <x:v>Machine-readable text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>indicator</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Stable machine-readable indicator name</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Do not translate in code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>indicator_zh</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>Chinese label matching the official source concept</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>Human-readable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>MOA 2024 Detail</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>Total/marine/freshwater or operational subgroup</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>Controls valid aggregation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>reported_value</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Numeric value as displayed on the official page</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Never overwrite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>reported_unit</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>Unit as displayed on the official page</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>Never overwrite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>normalization_multiplier</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Exact multiplier used for unit conversion</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>value = reported_value × multiplier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>all data sheets</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>Machine-readable normalized numeric value</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="str">
+        <x:v>Typed number</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>unit</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>all data sheets</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>Normalized unit</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>One unit per row</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>yoy_pct</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>MOA detail/latest</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>Signed year-on-year percent; declines are negative</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="str">
+        <x:v>Blank if source does not report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>share_pct</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>MOA 2024 Detail</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>Share reported in source table</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>Blank unless explicitly reported</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>comparison_year</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>Environment 2024</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>Baseline year for a change indicator</x:v>
+      </x:c>
+      <x:c r="D14" s="8" t="str">
+        <x:v>Do not treat changes as levels</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="8" t="str">
+        <x:v>change_direction</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>Environment 2024</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>level/increase/decrease classification</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="str">
+        <x:v>Interpret with comparison_year</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>category_basis</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>Latest Official</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>Production method or water-body basis</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="str">
+        <x:v>Do not combine unlike bases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>source_url</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>all data sheets</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>Official page or API URL</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>Plain-text auditable URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>source_sha256</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>SHA-256 of downloaded official HTML</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>64 lowercase hexadecimal characters</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="8" t="str">
+        <x:v>data_label</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>detailed/latest sheets</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>经过处理的数据（公开来源）</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>Never call author raw data</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>Relationship</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>Difference</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>Tolerance</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>MOA detailed row count</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>99 parsed records</x:v>
+      </x:c>
+      <x:c r="C2" s="24" t="n">
+        <x:f>COUNTA('MOA 2024 Detail'!A2:A100)-99</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D2" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
+        <x:f>IF(ABS(C2)&lt;=D2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>2024 economic output</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>total - fishery - industry/construction - circulation/services</x:v>
+      </x:c>
+      <x:c r="C3" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I61-'MOA 2024 Detail'!I55-'MOA 2024 Detail'!I54-'MOA 2024 Detail'!I53</x:f>
+        <x:v>1.8189894035458565e-12</x:v>
+      </x:c>
+      <x:c r="D3" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="str">
+        <x:f>IF(ABS(C3)&lt;=D3,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>2024 aquatic production</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>total - aquaculture - capture</x:v>
+      </x:c>
+      <x:c r="C4" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I100-'MOA 2024 Detail'!I94-'MOA 2024 Detail'!I96</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D4" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:f>IF(ABS(C4)&lt;=D4,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>2024 capture composition</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>capture - domestic capture - distant-water capture</x:v>
+      </x:c>
+      <x:c r="C5" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I96-'MOA 2024 Detail'!I35-'MOA 2024 Detail'!I97</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D5" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:f>IF(ABS(C5)&lt;=D5,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>2024 water-body composition</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>total - marine - freshwater</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I100-'MOA 2024 Detail'!I99-'MOA 2024 Detail'!I98</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str">
+        <x:f>IF(ABS(C6)&lt;=D6,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>Motorized fleet tonnage</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>motorized - production - auxiliary (rounding allowed)</x:v>
+      </x:c>
+      <x:c r="C7" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I71-'MOA 2024 Detail'!I73-'MOA 2024 Detail'!I70</x:f>
+        <x:v>-100</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:f>IF(ABS(C7)&lt;=D7,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>Processed products</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>total - marine - freshwater (rounding allowed)</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="n">
+        <x:f>'MOA 2024 Detail'!I82-'MOA 2024 Detail'!I81-'MOA 2024 Detail'!I80</x:f>
+        <x:v>3.725290298461914e-9</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:f>IF(ABS(C8)&lt;=D8,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>2025 China production</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>total - aquaculture - capture</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="n">
+        <x:f>'Latest Official'!I2-'Latest Official'!I3-'Latest Official'!I4</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="str">
+        <x:f>IF(ABS(C9)&lt;=D9,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>2025 Zhejiang production</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>total - marine - freshwater</x:v>
+      </x:c>
+      <x:c r="C10" s="24" t="n">
+        <x:f>'Latest Official'!I5-'Latest Official'!I6-'Latest Official'!I7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="E10" s="8" t="str">
+        <x:f>IF(ABS(C10)&lt;=D10,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>NBS province rows</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>31 official province-level rows</x:v>
+      </x:c>
+      <x:c r="C11" s="24" t="n">
+        <x:f>COUNTA('NBS 2024 Provinces'!A2:A32)-31</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:f>IF(ABS(C11)&lt;=D11,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>NBS 2024 aquatic total</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>province sum - printed national value</x:v>
+      </x:c>
+      <x:c r="C12" s="24" t="n">
+        <x:f>SUM('NBS 2024 Provinces'!E2:E32)-'NBS National QC'!B2</x:f>
+        <x:v>0.09999999999763531</x:v>
+      </x:c>
+      <x:c r="D12" s="24" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="E12" s="8" t="str">
+        <x:f>IF(ABS(C12)&lt;=D12,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>NBS 2024 freight scope</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>province sum + not-classified amount - printed national value</x:v>
+      </x:c>
+      <x:c r="C13" s="24" t="n">
+        <x:f>SUM('NBS 2024 Provinces'!P2:P32)+97072-'NBS National QC'!B13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="str">
+        <x:f>IF(ABS(C13)&lt;=D13,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>NBS 2024 e-commerce enterprises</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>province sum - printed national value</x:v>
+      </x:c>
+      <x:c r="C14" s="24" t="n">
+        <x:f>SUM('NBS 2024 Provinces'!R2:R32)-'NBS National QC'!B15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="8" t="str">
+        <x:f>IF(ABS(C14)&lt;=D14,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="E2:E14">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="FAIL"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -10519,6 +11248,3121 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="28" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="52" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="42" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>province_code</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>province_en</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>province_zh</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>aquatic_total_10000_t</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>marine_total_10000_t</x:v>
+      </x:c>
+      <x:c r="G1" s="12" t="str">
+        <x:v>marine_capture_10000_t</x:v>
+      </x:c>
+      <x:c r="H1" s="12" t="str">
+        <x:v>marine_aquaculture_10000_t</x:v>
+      </x:c>
+      <x:c r="I1" s="12" t="str">
+        <x:v>freshwater_total_10000_t</x:v>
+      </x:c>
+      <x:c r="J1" s="12" t="str">
+        <x:v>freshwater_capture_10000_t</x:v>
+      </x:c>
+      <x:c r="K1" s="12" t="str">
+        <x:v>freshwater_aquaculture_10000_t</x:v>
+      </x:c>
+      <x:c r="L1" s="12" t="str">
+        <x:v>population_10000_persons</x:v>
+      </x:c>
+      <x:c r="M1" s="12" t="str">
+        <x:v>disposable_income_yuan</x:v>
+      </x:c>
+      <x:c r="N1" s="12" t="str">
+        <x:v>wastewater_cod_tonnes</x:v>
+      </x:c>
+      <x:c r="O1" s="12" t="str">
+        <x:v>wastewater_total_phosphorus_tonnes</x:v>
+      </x:c>
+      <x:c r="P1" s="12" t="str">
+        <x:v>freight_total_10000_tonnes</x:v>
+      </x:c>
+      <x:c r="Q1" s="12" t="str">
+        <x:v>enterprises_units</x:v>
+      </x:c>
+      <x:c r="R1" s="12" t="str">
+        <x:v>ecommerce_enterprises_units</x:v>
+      </x:c>
+      <x:c r="S1" s="12" t="str">
+        <x:v>ecommerce_sales_100m_yuan</x:v>
+      </x:c>
+      <x:c r="T1" s="12" t="str">
+        <x:v>source_tables</x:v>
+      </x:c>
+      <x:c r="U1" s="12" t="str">
+        <x:v>data_status</x:v>
+      </x:c>
+      <x:c r="V1" s="12" t="str">
+        <x:v>transcription_note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>CN-BJ</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>Beijing</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>北京</x:v>
+      </x:c>
+      <x:c r="D2" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E2" s="22" t="n">
+        <x:v>7.1</x:v>
+      </x:c>
+      <x:c r="F2" s="22" t="n">
+        <x:v>5.7</x:v>
+      </x:c>
+      <x:c r="G2" s="22" t="n">
+        <x:v>5.7</x:v>
+      </x:c>
+      <x:c r="H2" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" s="22" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="J2" s="22" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="K2" s="22" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="L2" s="22" t="n">
+        <x:v>2183</x:v>
+      </x:c>
+      <x:c r="M2" s="22" t="n">
+        <x:v>85415</x:v>
+      </x:c>
+      <x:c r="N2" s="22" t="n">
+        <x:v>114599</x:v>
+      </x:c>
+      <x:c r="O2" s="22" t="n">
+        <x:v>1185</x:v>
+      </x:c>
+      <x:c r="P2" s="22" t="n">
+        <x:v>19956</x:v>
+      </x:c>
+      <x:c r="Q2" s="22" t="n">
+        <x:v>49504</x:v>
+      </x:c>
+      <x:c r="R2" s="22" t="n">
+        <x:v>11528</x:v>
+      </x:c>
+      <x:c r="S2" s="22" t="n">
+        <x:v>46980.2</x:v>
+      </x:c>
+      <x:c r="T2" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U2" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V2" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>CN-TJ</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>Tianjin</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>天津</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E3" s="22" t="n">
+        <x:v>29.9</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="G3" s="22" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="H3" s="22" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="I3" s="22" t="n">
+        <x:v>25.4</x:v>
+      </x:c>
+      <x:c r="J3" s="22" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="K3" s="22" t="n">
+        <x:v>25.1</x:v>
+      </x:c>
+      <x:c r="L3" s="22" t="n">
+        <x:v>1364</x:v>
+      </x:c>
+      <x:c r="M3" s="22" t="n">
+        <x:v>53581</x:v>
+      </x:c>
+      <x:c r="N3" s="22" t="n">
+        <x:v>189195</x:v>
+      </x:c>
+      <x:c r="O3" s="22" t="n">
+        <x:v>2054</x:v>
+      </x:c>
+      <x:c r="P3" s="22" t="n">
+        <x:v>58602</x:v>
+      </x:c>
+      <x:c r="Q3" s="22" t="n">
+        <x:v>29626</x:v>
+      </x:c>
+      <x:c r="R3" s="22" t="n">
+        <x:v>2619</x:v>
+      </x:c>
+      <x:c r="S3" s="22" t="n">
+        <x:v>8126.2</x:v>
+      </x:c>
+      <x:c r="T3" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U3" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V3" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>CN-HE</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Hebei</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>河北</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="F4" s="22" t="n">
+        <x:v>85.4</x:v>
+      </x:c>
+      <x:c r="G4" s="22" t="n">
+        <x:v>22.1</x:v>
+      </x:c>
+      <x:c r="H4" s="22" t="n">
+        <x:v>63.3</x:v>
+      </x:c>
+      <x:c r="I4" s="22" t="n">
+        <x:v>32.6</x:v>
+      </x:c>
+      <x:c r="J4" s="22" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="K4" s="22" t="n">
+        <x:v>28.1</x:v>
+      </x:c>
+      <x:c r="L4" s="22" t="n">
+        <x:v>7378</x:v>
+      </x:c>
+      <x:c r="M4" s="22" t="n">
+        <x:v>34665</x:v>
+      </x:c>
+      <x:c r="N4" s="22" t="n">
+        <x:v>1536069</x:v>
+      </x:c>
+      <x:c r="O4" s="22" t="n">
+        <x:v>16123</x:v>
+      </x:c>
+      <x:c r="P4" s="22" t="n">
+        <x:v>270712</x:v>
+      </x:c>
+      <x:c r="Q4" s="22" t="n">
+        <x:v>43022</x:v>
+      </x:c>
+      <x:c r="R4" s="22" t="n">
+        <x:v>3671</x:v>
+      </x:c>
+      <x:c r="S4" s="22" t="n">
+        <x:v>4056.8</x:v>
+      </x:c>
+      <x:c r="T4" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U4" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V4" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>CN-SX</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>Shanxi</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>山西</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
+        <x:v>5.8</x:v>
+      </x:c>
+      <x:c r="F5" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="22" t="n">
+        <x:v>5.8</x:v>
+      </x:c>
+      <x:c r="J5" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="n">
+        <x:v>5.8</x:v>
+      </x:c>
+      <x:c r="L5" s="22" t="n">
+        <x:v>3446</x:v>
+      </x:c>
+      <x:c r="M5" s="22" t="n">
+        <x:v>32441</x:v>
+      </x:c>
+      <x:c r="N5" s="22" t="n">
+        <x:v>793400</x:v>
+      </x:c>
+      <x:c r="O5" s="22" t="n">
+        <x:v>9288</x:v>
+      </x:c>
+      <x:c r="P5" s="22" t="n">
+        <x:v>224552</x:v>
+      </x:c>
+      <x:c r="Q5" s="22" t="n">
+        <x:v>28985</x:v>
+      </x:c>
+      <x:c r="R5" s="22" t="n">
+        <x:v>2600</x:v>
+      </x:c>
+      <x:c r="S5" s="22" t="n">
+        <x:v>6152.9</x:v>
+      </x:c>
+      <x:c r="T5" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U5" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V5" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>CN-NM</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>Inner Mongolia</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>内蒙古</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:v>11.6</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="n">
+        <x:v>10.4</x:v>
+      </x:c>
+      <x:c r="L6" s="22" t="n">
+        <x:v>2388</x:v>
+      </x:c>
+      <x:c r="M6" s="22" t="n">
+        <x:v>40077</x:v>
+      </x:c>
+      <x:c r="N6" s="22" t="n">
+        <x:v>906870</x:v>
+      </x:c>
+      <x:c r="O6" s="22" t="n">
+        <x:v>5604</x:v>
+      </x:c>
+      <x:c r="P6" s="22" t="n">
+        <x:v>251474</x:v>
+      </x:c>
+      <x:c r="Q6" s="22" t="n">
+        <x:v>13949</x:v>
+      </x:c>
+      <x:c r="R6" s="22" t="n">
+        <x:v>1521</x:v>
+      </x:c>
+      <x:c r="S6" s="22" t="n">
+        <x:v>6194.2</x:v>
+      </x:c>
+      <x:c r="T6" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U6" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V6" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>CN-LN</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Liaoning</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>辽宁</x:v>
+      </x:c>
+      <x:c r="D7" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>535.9</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="G7" s="22" t="n">
+        <x:v>69.7</x:v>
+      </x:c>
+      <x:c r="H7" s="22" t="n">
+        <x:v>382.3</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="n">
+        <x:v>83.9</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="n">
+        <x:v>80.6</x:v>
+      </x:c>
+      <x:c r="L7" s="22" t="n">
+        <x:v>4155</x:v>
+      </x:c>
+      <x:c r="M7" s="22" t="n">
+        <x:v>39844</x:v>
+      </x:c>
+      <x:c r="N7" s="22" t="n">
+        <x:v>1372012</x:v>
+      </x:c>
+      <x:c r="O7" s="22" t="n">
+        <x:v>15537</x:v>
+      </x:c>
+      <x:c r="P7" s="22" t="n">
+        <x:v>185682</x:v>
+      </x:c>
+      <x:c r="Q7" s="22" t="n">
+        <x:v>33151</x:v>
+      </x:c>
+      <x:c r="R7" s="22" t="n">
+        <x:v>2759</x:v>
+      </x:c>
+      <x:c r="S7" s="22" t="n">
+        <x:v>6954.6</x:v>
+      </x:c>
+      <x:c r="T7" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U7" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V7" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>CN-JL</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>Jilin</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>吉林</x:v>
+      </x:c>
+      <x:c r="D8" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>26.6</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="n">
+        <x:v>26.6</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="n">
+        <x:v>24.8</x:v>
+      </x:c>
+      <x:c r="L8" s="22" t="n">
+        <x:v>2317</x:v>
+      </x:c>
+      <x:c r="M8" s="22" t="n">
+        <x:v>31318</x:v>
+      </x:c>
+      <x:c r="N8" s="22" t="n">
+        <x:v>899449</x:v>
+      </x:c>
+      <x:c r="O8" s="22" t="n">
+        <x:v>7346</x:v>
+      </x:c>
+      <x:c r="P8" s="22" t="n">
+        <x:v>55578</x:v>
+      </x:c>
+      <x:c r="Q8" s="22" t="n">
+        <x:v>13240</x:v>
+      </x:c>
+      <x:c r="R8" s="22" t="n">
+        <x:v>1018</x:v>
+      </x:c>
+      <x:c r="S8" s="22" t="n">
+        <x:v>1322.6</x:v>
+      </x:c>
+      <x:c r="T8" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U8" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V8" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>CN-HL</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>Heilongjiang</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>黑龙江</x:v>
+      </x:c>
+      <x:c r="D9" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
+        <x:v>81.4</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="n">
+        <x:v>81.4</x:v>
+      </x:c>
+      <x:c r="J9" s="22" t="n">
+        <x:v>5.1</x:v>
+      </x:c>
+      <x:c r="K9" s="22" t="n">
+        <x:v>76.3</x:v>
+      </x:c>
+      <x:c r="L9" s="22" t="n">
+        <x:v>3029</x:v>
+      </x:c>
+      <x:c r="M9" s="22" t="n">
+        <x:v>31269</x:v>
+      </x:c>
+      <x:c r="N9" s="22" t="n">
+        <x:v>1004969</x:v>
+      </x:c>
+      <x:c r="O9" s="22" t="n">
+        <x:v>9166</x:v>
+      </x:c>
+      <x:c r="P9" s="22" t="n">
+        <x:v>55452</x:v>
+      </x:c>
+      <x:c r="Q9" s="22" t="n">
+        <x:v>15078</x:v>
+      </x:c>
+      <x:c r="R9" s="22" t="n">
+        <x:v>1263</x:v>
+      </x:c>
+      <x:c r="S9" s="22" t="n">
+        <x:v>1372.8</x:v>
+      </x:c>
+      <x:c r="T9" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U9" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V9" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>CN-SH</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>Shanghai</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>上海</x:v>
+      </x:c>
+      <x:c r="D10" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E10" s="22" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="n">
+        <x:v>12.1</x:v>
+      </x:c>
+      <x:c r="G10" s="22" t="n">
+        <x:v>12.1</x:v>
+      </x:c>
+      <x:c r="H10" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J10" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="22" t="n">
+        <x:v>9.9</x:v>
+      </x:c>
+      <x:c r="L10" s="22" t="n">
+        <x:v>2480</x:v>
+      </x:c>
+      <x:c r="M10" s="22" t="n">
+        <x:v>88366</x:v>
+      </x:c>
+      <x:c r="N10" s="22" t="n">
+        <x:v>130709</x:v>
+      </x:c>
+      <x:c r="O10" s="22" t="n">
+        <x:v>1617</x:v>
+      </x:c>
+      <x:c r="P10" s="22" t="n">
+        <x:v>155511</x:v>
+      </x:c>
+      <x:c r="Q10" s="22" t="n">
+        <x:v>57286</x:v>
+      </x:c>
+      <x:c r="R10" s="22" t="n">
+        <x:v>8479</x:v>
+      </x:c>
+      <x:c r="S10" s="22" t="n">
+        <x:v>46683.4</x:v>
+      </x:c>
+      <x:c r="T10" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U10" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V10" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>CN-JS</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Jiangsu</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>江苏</x:v>
+      </x:c>
+      <x:c r="D11" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:v>536.1</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="n">
+        <x:v>148.1</x:v>
+      </x:c>
+      <x:c r="G11" s="22" t="n">
+        <x:v>45.8</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="n">
+        <x:v>102.3</x:v>
+      </x:c>
+      <x:c r="I11" s="22" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="J11" s="22" t="n">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="K11" s="22" t="n">
+        <x:v>369.4</x:v>
+      </x:c>
+      <x:c r="L11" s="22" t="n">
+        <x:v>8526</x:v>
+      </x:c>
+      <x:c r="M11" s="22" t="n">
+        <x:v>55415</x:v>
+      </x:c>
+      <x:c r="N11" s="22" t="n">
+        <x:v>1206340</x:v>
+      </x:c>
+      <x:c r="O11" s="22" t="n">
+        <x:v>18831</x:v>
+      </x:c>
+      <x:c r="P11" s="22" t="n">
+        <x:v>319944</x:v>
+      </x:c>
+      <x:c r="Q11" s="22" t="n">
+        <x:v>185646</x:v>
+      </x:c>
+      <x:c r="R11" s="22" t="n">
+        <x:v>21199</x:v>
+      </x:c>
+      <x:c r="S11" s="22" t="n">
+        <x:v>30208.7</x:v>
+      </x:c>
+      <x:c r="T11" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U11" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V11" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>CN-ZJ</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Zhejiang</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>浙江</x:v>
+      </x:c>
+      <x:c r="D12" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E12" s="22" t="n">
+        <x:v>649.5</x:v>
+      </x:c>
+      <x:c r="F12" s="22" t="n">
+        <x:v>488.5</x:v>
+      </x:c>
+      <x:c r="G12" s="22" t="n">
+        <x:v>316.3</x:v>
+      </x:c>
+      <x:c r="H12" s="22" t="n">
+        <x:v>172.2</x:v>
+      </x:c>
+      <x:c r="I12" s="22" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="J12" s="22" t="n">
+        <x:v>17.1</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="L12" s="22" t="n">
+        <x:v>6670</x:v>
+      </x:c>
+      <x:c r="M12" s="22" t="n">
+        <x:v>67013</x:v>
+      </x:c>
+      <x:c r="N12" s="22" t="n">
+        <x:v>514440</x:v>
+      </x:c>
+      <x:c r="O12" s="22" t="n">
+        <x:v>12599</x:v>
+      </x:c>
+      <x:c r="P12" s="22" t="n">
+        <x:v>371158</x:v>
+      </x:c>
+      <x:c r="Q12" s="22" t="n">
+        <x:v>139433</x:v>
+      </x:c>
+      <x:c r="R12" s="22" t="n">
+        <x:v>19861</x:v>
+      </x:c>
+      <x:c r="S12" s="22" t="n">
+        <x:v>27311.2</x:v>
+      </x:c>
+      <x:c r="T12" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U12" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V12" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>CN-AH</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Anhui</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>安徽</x:v>
+      </x:c>
+      <x:c r="D13" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
+        <x:v>261.2</x:v>
+      </x:c>
+      <x:c r="F13" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="22" t="n">
+        <x:v>261.2</x:v>
+      </x:c>
+      <x:c r="J13" s="22" t="n">
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="K13" s="22" t="n">
+        <x:v>251.4</x:v>
+      </x:c>
+      <x:c r="L13" s="22" t="n">
+        <x:v>6123</x:v>
+      </x:c>
+      <x:c r="M13" s="22" t="n">
+        <x:v>36782</x:v>
+      </x:c>
+      <x:c r="N13" s="22" t="n">
+        <x:v>1397464</x:v>
+      </x:c>
+      <x:c r="O13" s="22" t="n">
+        <x:v>22504</x:v>
+      </x:c>
+      <x:c r="P13" s="22" t="n">
+        <x:v>441542</x:v>
+      </x:c>
+      <x:c r="Q13" s="22" t="n">
+        <x:v>58921</x:v>
+      </x:c>
+      <x:c r="R13" s="22" t="n">
+        <x:v>7057</x:v>
+      </x:c>
+      <x:c r="S13" s="22" t="n">
+        <x:v>11568.9</x:v>
+      </x:c>
+      <x:c r="T13" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U13" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V13" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>CN-FJ</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>Fujian</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>福建</x:v>
+      </x:c>
+      <x:c r="D14" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="n">
+        <x:v>924.7</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="n">
+        <x:v>818.7</x:v>
+      </x:c>
+      <x:c r="G14" s="22" t="n">
+        <x:v>205.4</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="n">
+        <x:v>613.3</x:v>
+      </x:c>
+      <x:c r="I14" s="22" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="n">
+        <x:v>7.3</x:v>
+      </x:c>
+      <x:c r="K14" s="22" t="n">
+        <x:v>98.7</x:v>
+      </x:c>
+      <x:c r="L14" s="22" t="n">
+        <x:v>4193</x:v>
+      </x:c>
+      <x:c r="M14" s="22" t="n">
+        <x:v>47857</x:v>
+      </x:c>
+      <x:c r="N14" s="22" t="n">
+        <x:v>602380</x:v>
+      </x:c>
+      <x:c r="O14" s="22" t="n">
+        <x:v>15302</x:v>
+      </x:c>
+      <x:c r="P14" s="22" t="n">
+        <x:v>183536</x:v>
+      </x:c>
+      <x:c r="Q14" s="22" t="n">
+        <x:v>73324</x:v>
+      </x:c>
+      <x:c r="R14" s="22" t="n">
+        <x:v>9134</x:v>
+      </x:c>
+      <x:c r="S14" s="22" t="n">
+        <x:v>13504.5</x:v>
+      </x:c>
+      <x:c r="T14" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U14" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V14" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="8" t="str">
+        <x:v>CN-JX</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>Jiangxi</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>江西</x:v>
+      </x:c>
+      <x:c r="D15" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
+        <x:v>303.3</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="22" t="n">
+        <x:v>303.3</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K15" s="22" t="n">
+        <x:v>302.2</x:v>
+      </x:c>
+      <x:c r="L15" s="22" t="n">
+        <x:v>4502</x:v>
+      </x:c>
+      <x:c r="M15" s="22" t="n">
+        <x:v>36007</x:v>
+      </x:c>
+      <x:c r="N15" s="22" t="n">
+        <x:v>1044465</x:v>
+      </x:c>
+      <x:c r="O15" s="22" t="n">
+        <x:v>17393</x:v>
+      </x:c>
+      <x:c r="P15" s="22" t="n">
+        <x:v>215859</x:v>
+      </x:c>
+      <x:c r="Q15" s="22" t="n">
+        <x:v>54180</x:v>
+      </x:c>
+      <x:c r="R15" s="22" t="n">
+        <x:v>6792</x:v>
+      </x:c>
+      <x:c r="S15" s="22" t="n">
+        <x:v>4765.4</x:v>
+      </x:c>
+      <x:c r="T15" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U15" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V15" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>CN-SD</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>Shandong</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>山东</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E16" s="22" t="n">
+        <x:v>952.7</x:v>
+      </x:c>
+      <x:c r="F16" s="22" t="n">
+        <x:v>825.2</x:v>
+      </x:c>
+      <x:c r="G16" s="22" t="n">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="H16" s="22" t="n">
+        <x:v>606.3</x:v>
+      </x:c>
+      <x:c r="I16" s="22" t="n">
+        <x:v>127.5</x:v>
+      </x:c>
+      <x:c r="J16" s="22" t="n">
+        <x:v>10.8</x:v>
+      </x:c>
+      <x:c r="K16" s="22" t="n">
+        <x:v>116.7</x:v>
+      </x:c>
+      <x:c r="L16" s="22" t="n">
+        <x:v>10080</x:v>
+      </x:c>
+      <x:c r="M16" s="22" t="n">
+        <x:v>42077</x:v>
+      </x:c>
+      <x:c r="N16" s="22" t="n">
+        <x:v>1542184</x:v>
+      </x:c>
+      <x:c r="O16" s="22" t="n">
+        <x:v>16048</x:v>
+      </x:c>
+      <x:c r="P16" s="22" t="n">
+        <x:v>355666</x:v>
+      </x:c>
+      <x:c r="Q16" s="22" t="n">
+        <x:v>128344</x:v>
+      </x:c>
+      <x:c r="R16" s="22" t="n">
+        <x:v>21871</x:v>
+      </x:c>
+      <x:c r="S16" s="22" t="n">
+        <x:v>34535.2</x:v>
+      </x:c>
+      <x:c r="T16" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U16" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V16" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>CN-HA</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>Henan</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>河南</x:v>
+      </x:c>
+      <x:c r="D17" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
+        <x:v>100.4</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="22" t="n">
+        <x:v>100.4</x:v>
+      </x:c>
+      <x:c r="J17" s="22" t="n">
+        <x:v>11.1</x:v>
+      </x:c>
+      <x:c r="K17" s="22" t="n">
+        <x:v>89.3</x:v>
+      </x:c>
+      <x:c r="L17" s="22" t="n">
+        <x:v>9785</x:v>
+      </x:c>
+      <x:c r="M17" s="22" t="n">
+        <x:v>31552</x:v>
+      </x:c>
+      <x:c r="N17" s="22" t="n">
+        <x:v>1699957</x:v>
+      </x:c>
+      <x:c r="O17" s="22" t="n">
+        <x:v>21009</x:v>
+      </x:c>
+      <x:c r="P17" s="22" t="n">
+        <x:v>293441</x:v>
+      </x:c>
+      <x:c r="Q17" s="22" t="n">
+        <x:v>75879</x:v>
+      </x:c>
+      <x:c r="R17" s="22" t="n">
+        <x:v>6797</x:v>
+      </x:c>
+      <x:c r="S17" s="22" t="n">
+        <x:v>9664.9</x:v>
+      </x:c>
+      <x:c r="T17" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U17" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V17" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>CN-HB</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>Hubei</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>湖北</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E18" s="22" t="n">
+        <x:v>546.4</x:v>
+      </x:c>
+      <x:c r="F18" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="22" t="n">
+        <x:v>546.4</x:v>
+      </x:c>
+      <x:c r="J18" s="22" t="n">
+        <x:v>2.4</x:v>
+      </x:c>
+      <x:c r="K18" s="22" t="n">
+        <x:v>544.1</x:v>
+      </x:c>
+      <x:c r="L18" s="22" t="n">
+        <x:v>5834</x:v>
+      </x:c>
+      <x:c r="M18" s="22" t="n">
+        <x:v>36947</x:v>
+      </x:c>
+      <x:c r="N18" s="22" t="n">
+        <x:v>1490235</x:v>
+      </x:c>
+      <x:c r="O18" s="22" t="n">
+        <x:v>24650</x:v>
+      </x:c>
+      <x:c r="P18" s="22" t="n">
+        <x:v>267173</x:v>
+      </x:c>
+      <x:c r="Q18" s="22" t="n">
+        <x:v>70736</x:v>
+      </x:c>
+      <x:c r="R18" s="22" t="n">
+        <x:v>9377</x:v>
+      </x:c>
+      <x:c r="S18" s="22" t="n">
+        <x:v>10974.4</x:v>
+      </x:c>
+      <x:c r="T18" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U18" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V18" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="8" t="str">
+        <x:v>CN-HN</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>Hunan</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>湖南</x:v>
+      </x:c>
+      <x:c r="D19" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
+        <x:v>299.1</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="22" t="n">
+        <x:v>299.1</x:v>
+      </x:c>
+      <x:c r="J19" s="22" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="n">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="L19" s="22" t="n">
+        <x:v>6539</x:v>
+      </x:c>
+      <x:c r="M19" s="22" t="n">
+        <x:v>37679</x:v>
+      </x:c>
+      <x:c r="N19" s="22" t="n">
+        <x:v>1732340</x:v>
+      </x:c>
+      <x:c r="O19" s="22" t="n">
+        <x:v>28663</x:v>
+      </x:c>
+      <x:c r="P19" s="22" t="n">
+        <x:v>237819</x:v>
+      </x:c>
+      <x:c r="Q19" s="22" t="n">
+        <x:v>56846</x:v>
+      </x:c>
+      <x:c r="R19" s="22" t="n">
+        <x:v>7094</x:v>
+      </x:c>
+      <x:c r="S19" s="22" t="n">
+        <x:v>6560.1</x:v>
+      </x:c>
+      <x:c r="T19" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U19" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V19" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="8" t="str">
+        <x:v>CN-GD</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>Guangdong</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>广东</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="n">
+        <x:v>966.4</x:v>
+      </x:c>
+      <x:c r="F20" s="22" t="n">
+        <x:v>508.4</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
+        <x:v>131.5</x:v>
+      </x:c>
+      <x:c r="H20" s="22" t="n">
+        <x:v>376.8</x:v>
+      </x:c>
+      <x:c r="I20" s="22" t="n">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="J20" s="22" t="n">
+        <x:v>7.2</x:v>
+      </x:c>
+      <x:c r="K20" s="22" t="n">
+        <x:v>450.8</x:v>
+      </x:c>
+      <x:c r="L20" s="22" t="n">
+        <x:v>12780</x:v>
+      </x:c>
+      <x:c r="M20" s="22" t="n">
+        <x:v>51474</x:v>
+      </x:c>
+      <x:c r="N20" s="22" t="n">
+        <x:v>1706500</x:v>
+      </x:c>
+      <x:c r="O20" s="22" t="n">
+        <x:v>33917</x:v>
+      </x:c>
+      <x:c r="P20" s="22" t="n">
+        <x:v>371959</x:v>
+      </x:c>
+      <x:c r="Q20" s="22" t="n">
+        <x:v>215442</x:v>
+      </x:c>
+      <x:c r="R20" s="22" t="n">
+        <x:v>27520</x:v>
+      </x:c>
+      <x:c r="S20" s="22" t="n">
+        <x:v>53706.6</x:v>
+      </x:c>
+      <x:c r="T20" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U20" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V20" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="8" t="str">
+        <x:v>CN-GX</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>Guangxi</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>广西</x:v>
+      </x:c>
+      <x:c r="D21" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>388.7</x:v>
+      </x:c>
+      <x:c r="F21" s="22" t="n">
+        <x:v>228.4</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
+        <x:v>49.2</x:v>
+      </x:c>
+      <x:c r="H21" s="22" t="n">
+        <x:v>179.3</x:v>
+      </x:c>
+      <x:c r="I21" s="22" t="n">
+        <x:v>160.2</x:v>
+      </x:c>
+      <x:c r="J21" s="22" t="n">
+        <x:v>7.6</x:v>
+      </x:c>
+      <x:c r="K21" s="22" t="n">
+        <x:v>152.6</x:v>
+      </x:c>
+      <x:c r="L21" s="22" t="n">
+        <x:v>5013</x:v>
+      </x:c>
+      <x:c r="M21" s="22" t="n">
+        <x:v>31125</x:v>
+      </x:c>
+      <x:c r="N21" s="22" t="n">
+        <x:v>1005915</x:v>
+      </x:c>
+      <x:c r="O21" s="22" t="n">
+        <x:v>25624</x:v>
+      </x:c>
+      <x:c r="P21" s="22" t="n">
+        <x:v>237126</x:v>
+      </x:c>
+      <x:c r="Q21" s="22" t="n">
+        <x:v>29995</x:v>
+      </x:c>
+      <x:c r="R21" s="22" t="n">
+        <x:v>3393</x:v>
+      </x:c>
+      <x:c r="S21" s="22" t="n">
+        <x:v>4789.4</x:v>
+      </x:c>
+      <x:c r="T21" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U21" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V21" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="8" t="str">
+        <x:v>CN-HI</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>Hainan</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>海南</x:v>
+      </x:c>
+      <x:c r="D22" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>181.4</x:v>
+      </x:c>
+      <x:c r="F22" s="22" t="n">
+        <x:v>131.9</x:v>
+      </x:c>
+      <x:c r="G22" s="22" t="n">
+        <x:v>101.3</x:v>
+      </x:c>
+      <x:c r="H22" s="22" t="n">
+        <x:v>30.6</x:v>
+      </x:c>
+      <x:c r="I22" s="22" t="n">
+        <x:v>49.5</x:v>
+      </x:c>
+      <x:c r="J22" s="22" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="K22" s="22" t="n">
+        <x:v>48.4</x:v>
+      </x:c>
+      <x:c r="L22" s="22" t="n">
+        <x:v>1048</x:v>
+      </x:c>
+      <x:c r="M22" s="22" t="n">
+        <x:v>34829</x:v>
+      </x:c>
+      <x:c r="N22" s="22" t="n">
+        <x:v>175979</x:v>
+      </x:c>
+      <x:c r="O22" s="22" t="n">
+        <x:v>4385</x:v>
+      </x:c>
+      <x:c r="P22" s="22" t="n">
+        <x:v>39138</x:v>
+      </x:c>
+      <x:c r="Q22" s="22" t="n">
+        <x:v>7496</x:v>
+      </x:c>
+      <x:c r="R22" s="22" t="n">
+        <x:v>1115</x:v>
+      </x:c>
+      <x:c r="S22" s="22" t="n">
+        <x:v>2983.1</x:v>
+      </x:c>
+      <x:c r="T22" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U22" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V22" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="8" t="str">
+        <x:v>CN-CQ</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>Chongqing</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>重庆</x:v>
+      </x:c>
+      <x:c r="D23" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>61.2</x:v>
+      </x:c>
+      <x:c r="F23" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="22" t="n">
+        <x:v>61.2</x:v>
+      </x:c>
+      <x:c r="J23" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K23" s="22" t="n">
+        <x:v>61.2</x:v>
+      </x:c>
+      <x:c r="L23" s="22" t="n">
+        <x:v>3190</x:v>
+      </x:c>
+      <x:c r="M23" s="22" t="n">
+        <x:v>39713</x:v>
+      </x:c>
+      <x:c r="N23" s="22" t="n">
+        <x:v>429462</x:v>
+      </x:c>
+      <x:c r="O23" s="22" t="n">
+        <x:v>6565</x:v>
+      </x:c>
+      <x:c r="P23" s="22" t="n">
+        <x:v>137534</x:v>
+      </x:c>
+      <x:c r="Q23" s="22" t="n">
+        <x:v>28526</x:v>
+      </x:c>
+      <x:c r="R23" s="22" t="n">
+        <x:v>4849</x:v>
+      </x:c>
+      <x:c r="S23" s="22" t="n">
+        <x:v>12395.5</x:v>
+      </x:c>
+      <x:c r="T23" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U23" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V23" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="8" t="str">
+        <x:v>CN-SC</x:v>
+      </x:c>
+      <x:c r="B24" s="8" t="str">
+        <x:v>Sichuan</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="str">
+        <x:v>四川</x:v>
+      </x:c>
+      <x:c r="D24" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>187.2</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="22" t="n">
+        <x:v>187.2</x:v>
+      </x:c>
+      <x:c r="J24" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="22" t="n">
+        <x:v>187.2</x:v>
+      </x:c>
+      <x:c r="L24" s="22" t="n">
+        <x:v>8364</x:v>
+      </x:c>
+      <x:c r="M24" s="22" t="n">
+        <x:v>34325</x:v>
+      </x:c>
+      <x:c r="N24" s="22" t="n">
+        <x:v>1473764</x:v>
+      </x:c>
+      <x:c r="O24" s="22" t="n">
+        <x:v>21037</x:v>
+      </x:c>
+      <x:c r="P24" s="22" t="n">
+        <x:v>206296</x:v>
+      </x:c>
+      <x:c r="Q24" s="22" t="n">
+        <x:v>69448</x:v>
+      </x:c>
+      <x:c r="R24" s="22" t="n">
+        <x:v>9132</x:v>
+      </x:c>
+      <x:c r="S24" s="22" t="n">
+        <x:v>12342.5</x:v>
+      </x:c>
+      <x:c r="T24" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U24" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V24" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="8" t="str">
+        <x:v>CN-GZ</x:v>
+      </x:c>
+      <x:c r="B25" s="8" t="str">
+        <x:v>Guizhou</x:v>
+      </x:c>
+      <x:c r="C25" s="8" t="str">
+        <x:v>贵州</x:v>
+      </x:c>
+      <x:c r="D25" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>29.5</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="22" t="n">
+        <x:v>29.5</x:v>
+      </x:c>
+      <x:c r="J25" s="22" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="K25" s="22" t="n">
+        <x:v>29.1</x:v>
+      </x:c>
+      <x:c r="L25" s="22" t="n">
+        <x:v>3860</x:v>
+      </x:c>
+      <x:c r="M25" s="22" t="n">
+        <x:v>28561</x:v>
+      </x:c>
+      <x:c r="N25" s="22" t="n">
+        <x:v>1179543</x:v>
+      </x:c>
+      <x:c r="O25" s="22" t="n">
+        <x:v>15993</x:v>
+      </x:c>
+      <x:c r="P25" s="22" t="n">
+        <x:v>113446</x:v>
+      </x:c>
+      <x:c r="Q25" s="22" t="n">
+        <x:v>19832</x:v>
+      </x:c>
+      <x:c r="R25" s="22" t="n">
+        <x:v>2371</x:v>
+      </x:c>
+      <x:c r="S25" s="22" t="n">
+        <x:v>5613.9</x:v>
+      </x:c>
+      <x:c r="T25" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U25" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V25" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="8" t="str">
+        <x:v>CN-YN</x:v>
+      </x:c>
+      <x:c r="B26" s="8" t="str">
+        <x:v>Yunnan</x:v>
+      </x:c>
+      <x:c r="C26" s="8" t="str">
+        <x:v>云南</x:v>
+      </x:c>
+      <x:c r="D26" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F26" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H26" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="22" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="J26" s="22" t="n">
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="K26" s="22" t="n">
+        <x:v>69.2</x:v>
+      </x:c>
+      <x:c r="L26" s="22" t="n">
+        <x:v>4655</x:v>
+      </x:c>
+      <x:c r="M26" s="22" t="n">
+        <x:v>29932</x:v>
+      </x:c>
+      <x:c r="N26" s="22" t="n">
+        <x:v>772366</x:v>
+      </x:c>
+      <x:c r="O26" s="22" t="n">
+        <x:v>12081</x:v>
+      </x:c>
+      <x:c r="P26" s="22" t="n">
+        <x:v>149114</x:v>
+      </x:c>
+      <x:c r="Q26" s="22" t="n">
+        <x:v>26807</x:v>
+      </x:c>
+      <x:c r="R26" s="22" t="n">
+        <x:v>3302</x:v>
+      </x:c>
+      <x:c r="S26" s="22" t="n">
+        <x:v>2774.5</x:v>
+      </x:c>
+      <x:c r="T26" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U26" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V26" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="8" t="str">
+        <x:v>CN-XZ</x:v>
+      </x:c>
+      <x:c r="B27" s="8" t="str">
+        <x:v>Tibet</x:v>
+      </x:c>
+      <x:c r="C27" s="8" t="str">
+        <x:v>西藏</x:v>
+      </x:c>
+      <x:c r="D27" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E27" s="22" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F27" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H27" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="22" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="J27" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K27" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L27" s="22" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="M27" s="22" t="n">
+        <x:v>31358</x:v>
+      </x:c>
+      <x:c r="N27" s="22" t="n">
+        <x:v>506406</x:v>
+      </x:c>
+      <x:c r="O27" s="22" t="n">
+        <x:v>4228</x:v>
+      </x:c>
+      <x:c r="P27" s="22" t="n">
+        <x:v>5167</x:v>
+      </x:c>
+      <x:c r="Q27" s="22" t="n">
+        <x:v>2440</x:v>
+      </x:c>
+      <x:c r="R27" s="22" t="n">
+        <x:v>278</x:v>
+      </x:c>
+      <x:c r="S27" s="22" t="n">
+        <x:v>295.4</x:v>
+      </x:c>
+      <x:c r="T27" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U27" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V27" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="8" t="str">
+        <x:v>CN-SN</x:v>
+      </x:c>
+      <x:c r="B28" s="8" t="str">
+        <x:v>Shaanxi</x:v>
+      </x:c>
+      <x:c r="C28" s="8" t="str">
+        <x:v>陕西</x:v>
+      </x:c>
+      <x:c r="D28" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E28" s="22" t="n">
+        <x:v>18.7</x:v>
+      </x:c>
+      <x:c r="F28" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H28" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="22" t="n">
+        <x:v>18.7</x:v>
+      </x:c>
+      <x:c r="J28" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="22" t="n">
+        <x:v>18.7</x:v>
+      </x:c>
+      <x:c r="L28" s="22" t="n">
+        <x:v>3953</x:v>
+      </x:c>
+      <x:c r="M28" s="22" t="n">
+        <x:v>33905</x:v>
+      </x:c>
+      <x:c r="N28" s="22" t="n">
+        <x:v>400614</x:v>
+      </x:c>
+      <x:c r="O28" s="22" t="n">
+        <x:v>4706</x:v>
+      </x:c>
+      <x:c r="P28" s="22" t="n">
+        <x:v>188371</x:v>
+      </x:c>
+      <x:c r="Q28" s="22" t="n">
+        <x:v>34025</x:v>
+      </x:c>
+      <x:c r="R28" s="22" t="n">
+        <x:v>4165</x:v>
+      </x:c>
+      <x:c r="S28" s="22" t="n">
+        <x:v>6857.4</x:v>
+      </x:c>
+      <x:c r="T28" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U28" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V28" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="8" t="str">
+        <x:v>CN-GS</x:v>
+      </x:c>
+      <x:c r="B29" s="8" t="str">
+        <x:v>Gansu</x:v>
+      </x:c>
+      <x:c r="C29" s="8" t="str">
+        <x:v>甘肃</x:v>
+      </x:c>
+      <x:c r="D29" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E29" s="22" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="F29" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H29" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="22" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="J29" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="22" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="L29" s="22" t="n">
+        <x:v>2458</x:v>
+      </x:c>
+      <x:c r="M29" s="22" t="n">
+        <x:v>26612</x:v>
+      </x:c>
+      <x:c r="N29" s="22" t="n">
+        <x:v>920791</x:v>
+      </x:c>
+      <x:c r="O29" s="22" t="n">
+        <x:v>6804</x:v>
+      </x:c>
+      <x:c r="P29" s="22" t="n">
+        <x:v>84024</x:v>
+      </x:c>
+      <x:c r="Q29" s="22" t="n">
+        <x:v>14002</x:v>
+      </x:c>
+      <x:c r="R29" s="22" t="n">
+        <x:v>1391</x:v>
+      </x:c>
+      <x:c r="S29" s="22" t="n">
+        <x:v>1576.3</x:v>
+      </x:c>
+      <x:c r="T29" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U29" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V29" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="8" t="str">
+        <x:v>CN-QH</x:v>
+      </x:c>
+      <x:c r="B30" s="8" t="str">
+        <x:v>Qinghai</x:v>
+      </x:c>
+      <x:c r="C30" s="8" t="str">
+        <x:v>青海</x:v>
+      </x:c>
+      <x:c r="D30" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="n">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="F30" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="22" t="n">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="J30" s="22" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="K30" s="22" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="L30" s="22" t="n">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="M30" s="22" t="n">
+        <x:v>30117</x:v>
+      </x:c>
+      <x:c r="N30" s="22" t="n">
+        <x:v>281929</x:v>
+      </x:c>
+      <x:c r="O30" s="22" t="n">
+        <x:v>1456</x:v>
+      </x:c>
+      <x:c r="P30" s="22" t="n">
+        <x:v>21137</x:v>
+      </x:c>
+      <x:c r="Q30" s="22" t="n">
+        <x:v>3147</x:v>
+      </x:c>
+      <x:c r="R30" s="22" t="n">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="S30" s="22" t="n">
+        <x:v>380.8</x:v>
+      </x:c>
+      <x:c r="T30" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U30" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V30" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="8" t="str">
+        <x:v>CN-NX</x:v>
+      </x:c>
+      <x:c r="B31" s="8" t="str">
+        <x:v>Ningxia</x:v>
+      </x:c>
+      <x:c r="C31" s="8" t="str">
+        <x:v>宁夏</x:v>
+      </x:c>
+      <x:c r="D31" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E31" s="22" t="n">
+        <x:v>17.9</x:v>
+      </x:c>
+      <x:c r="F31" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="22" t="n">
+        <x:v>17.9</x:v>
+      </x:c>
+      <x:c r="J31" s="22" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="K31" s="22" t="n">
+        <x:v>17.2</x:v>
+      </x:c>
+      <x:c r="L31" s="22" t="n">
+        <x:v>729</x:v>
+      </x:c>
+      <x:c r="M31" s="22" t="n">
+        <x:v>33355</x:v>
+      </x:c>
+      <x:c r="N31" s="22" t="n">
+        <x:v>263736</x:v>
+      </x:c>
+      <x:c r="O31" s="22" t="n">
+        <x:v>2469</x:v>
+      </x:c>
+      <x:c r="P31" s="22" t="n">
+        <x:v>57966</x:v>
+      </x:c>
+      <x:c r="Q31" s="22" t="n">
+        <x:v>4903</x:v>
+      </x:c>
+      <x:c r="R31" s="22" t="n">
+        <x:v>541</x:v>
+      </x:c>
+      <x:c r="S31" s="22" t="n">
+        <x:v>1015.2</x:v>
+      </x:c>
+      <x:c r="T31" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U31" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V31" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="8" t="str">
+        <x:v>CN-XJ</x:v>
+      </x:c>
+      <x:c r="B32" s="8" t="str">
+        <x:v>Xinjiang</x:v>
+      </x:c>
+      <x:c r="C32" s="8" t="str">
+        <x:v>新疆</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="n">
+        <x:v>19.3</x:v>
+      </x:c>
+      <x:c r="F32" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="22" t="n">
+        <x:v>19.3</x:v>
+      </x:c>
+      <x:c r="J32" s="22" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="K32" s="22" t="n">
+        <x:v>17.9</x:v>
+      </x:c>
+      <x:c r="L32" s="22" t="n">
+        <x:v>2623</x:v>
+      </x:c>
+      <x:c r="M32" s="22" t="n">
+        <x:v>30899</x:v>
+      </x:c>
+      <x:c r="N32" s="22" t="n">
+        <x:v>704744</x:v>
+      </x:c>
+      <x:c r="O32" s="22" t="n">
+        <x:v>6294</x:v>
+      </x:c>
+      <x:c r="P32" s="22" t="n">
+        <x:v>111618</x:v>
+      </x:c>
+      <x:c r="Q32" s="22" t="n">
+        <x:v>22133</x:v>
+      </x:c>
+      <x:c r="R32" s="22" t="n">
+        <x:v>1970</x:v>
+      </x:c>
+      <x:c r="S32" s="22" t="n">
+        <x:v>4876.2</x:v>
+      </x:c>
+      <x:c r="T32" s="8" t="str">
+        <x:v>NBS 2025 Tables 2-5; 6-18; 8-10; 12-15; 16-13; 16-39</x:v>
+      </x:c>
+      <x:c r="U32" s="8" t="str">
+        <x:v>official public data; manually transcribed and double-checked</x:v>
+      </x:c>
+      <x:c r="V32" s="8" t="str">
+        <x:v>Values retain the units printed by NBS; component totals can differ by 0.1 because the source is rounded to one decimal place.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="66" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="64" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>field</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>definition</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>unit</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>evidence_class</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>source_table</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>source_url</x:v>
+      </x:c>
+      <x:c r="G1" s="12" t="str">
+        <x:v>processing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>province_code</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>ISO-style subdivision code</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>identifier</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
+        <x:v>NBS tables</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/left_.htm</x:v>
+      </x:c>
+      <x:c r="G2" s="8" t="str">
+        <x:v>Assigned consistently across the six transcribed tables.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>province_en</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>Province-level region name in English</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="str">
+        <x:v>NBS tables</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/left_.htm</x:v>
+      </x:c>
+      <x:c r="G3" s="8" t="str">
+        <x:v>Transcribed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>province_zh</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Province-level region name in Chinese</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>identifier</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>NBS tables</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/left_.htm</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>Standard Chinese name added for usability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>Reference year</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:v>NBS tables</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/left_.htm</x:v>
+      </x:c>
+      <x:c r="G5" s="8" t="str">
+        <x:v>All included observations refer to 2024.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>aquatic_total_10000_t</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>Total output of aquatic products</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G6" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>marine_total_10000_t</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Output of marine aquatic products</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>marine_capture_10000_t</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>Output of marine fishing products</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G8" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>marine_aquaculture_10000_t</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>Output of marine aquacultural products</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>freshwater_total_10000_t</x:v>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
+        <x:v>Output of freshwater aquatic products</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E10" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G10" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>freshwater_capture_10000_t</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Output of freshwater fishing products</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>freshwater_aquaculture_10000_t</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Output of freshwater aquacultural products</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E12" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F12" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G12" s="8" t="str">
+        <x:v>Transcribed without changing the printed unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>population_10000_persons</x:v>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Population at year-end by region</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>10 000 persons</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="str">
+        <x:v>2-5 Population at Year-end by Region</x:v>
+      </x:c>
+      <x:c r="F13" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E02-05.jpg</x:v>
+      </x:c>
+      <x:c r="G13" s="8" t="str">
+        <x:v>2024 column transcribed; provincial sum excludes military personnel included in the national total.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>disposable_income_yuan</x:v>
+      </x:c>
+      <x:c r="B14" s="8" t="str">
+        <x:v>Per-capita disposable income of households</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>yuan per person</x:v>
+      </x:c>
+      <x:c r="D14" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E14" s="8" t="str">
+        <x:v>6-18 Per Capita Disposable Income of Households by Region</x:v>
+      </x:c>
+      <x:c r="F14" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E06-18.jpg</x:v>
+      </x:c>
+      <x:c r="G14" s="8" t="str">
+        <x:v>2024 column transcribed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="8" t="str">
+        <x:v>wastewater_cod_tonnes</x:v>
+      </x:c>
+      <x:c r="B15" s="8" t="str">
+        <x:v>Chemical oxygen demand discharged in wastewater</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>tonnes</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E15" s="8" t="str">
+        <x:v>8-10 Main Pollutant Contents Discharged in Wastewater by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F15" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E08-10.jpg</x:v>
+      </x:c>
+      <x:c r="G15" s="8" t="str">
+        <x:v>Transcribed; NBS marks this table as preliminary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>wastewater_total_phosphorus_tonnes</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>Total phosphorus discharged in wastewater</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>tonnes</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E16" s="8" t="str">
+        <x:v>8-10 Main Pollutant Contents Discharged in Wastewater by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F16" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E08-10.jpg</x:v>
+      </x:c>
+      <x:c r="G16" s="8" t="str">
+        <x:v>Transcribed; NBS marks this table as preliminary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="8" t="str">
+        <x:v>freight_total_10000_tonnes</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>Total freight traffic by region</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E17" s="8" t="str">
+        <x:v>16-13 Freight Traffic by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F17" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-13.jpg</x:v>
+      </x:c>
+      <x:c r="G17" s="8" t="str">
+        <x:v>Transcribed; the national total also includes freight not classified by region.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>enterprises_units</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>Number of enterprises</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E18" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F18" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G18" s="8" t="str">
+        <x:v>Transcribed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="8" t="str">
+        <x:v>ecommerce_enterprises_units</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>Enterprises with e-commerce transactions</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E19" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F19" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G19" s="8" t="str">
+        <x:v>Transcribed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="8" t="str">
+        <x:v>ecommerce_sales_100m_yuan</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>Sales of enterprises through e-commerce</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>100 million yuan</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>official public data</x:v>
+      </x:c>
+      <x:c r="E20" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F20" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G20" s="8" t="str">
+        <x:v>Transcribed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="8" t="str">
+        <x:v>data_status</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>Evidence classification</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>provenance control</x:v>
+      </x:c>
+      <x:c r="E21" s="8" t="str">
+        <x:v>Repository classification</x:v>
+      </x:c>
+      <x:c r="F21" s="8" t="str"/>
+      <x:c r="G21" s="8" t="str">
+        <x:v>All rows state that they are official public data and manual transcriptions; they are not historical author inputs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="8" t="str">
+        <x:v>transcription_note</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>Rounding and transcription qualification</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D22" s="8" t="str">
+        <x:v>provenance control</x:v>
+      </x:c>
+      <x:c r="E22" s="8" t="str">
+        <x:v>Repository classification</x:v>
+      </x:c>
+      <x:c r="F22" s="8" t="str"/>
+      <x:c r="G22" s="8" t="str">
+        <x:v>No interpolation or third-party value substitution.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="50" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="64" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>metric</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>unit</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="E1" s="12" t="str">
+        <x:v>source_table</x:v>
+      </x:c>
+      <x:c r="F1" s="12" t="str">
+        <x:v>source_url</x:v>
+      </x:c>
+      <x:c r="G1" s="12" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="8" t="str">
+        <x:v>aquatic_total</x:v>
+      </x:c>
+      <x:c r="B2" s="22" t="n">
+        <x:v>7357.6</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G2" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
+      <x:c r="A3" s="8" t="str">
+        <x:v>marine_total</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="n">
+        <x:v>3708.9</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G3" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="42" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>marine_capture</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="n">
+        <x:v>1181.2</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="8" t="str">
+        <x:v>marine_aquaculture</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="n">
+        <x:v>2527.6</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G5" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>freshwater_total</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="n">
+        <x:v>3648.7</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G6" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>freshwater_capture</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="n">
+        <x:v>116.3</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>freshwater_aquaculture</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="n">
+        <x:v>3532.4</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>12-15 Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="G8" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="8" t="str">
+        <x:v>population</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="n">
+        <x:v>140828</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>10 000 persons</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="str">
+        <x:v>2-5 Population at Year-end by Region</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E02-05.jpg</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="str">
+        <x:v>Includes military personnel excluded from provincial rows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="8" t="str">
+        <x:v>disposable_income</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="n">
+        <x:v>41314</x:v>
+      </x:c>
+      <x:c r="C10" s="8" t="str">
+        <x:v>yuan per person</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E10" s="8" t="str">
+        <x:v>6-18 Per Capita Disposable Income of Households by Region</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E06-18.jpg</x:v>
+      </x:c>
+      <x:c r="G10" s="8" t="str">
+        <x:v>National average; it is not the arithmetic mean of provincial values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>wastewater_cod</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="n">
+        <x:v>27998827</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>tonnes</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:v>8-10 Main Pollutant Contents Discharged in Wastewater by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E08-10.jpg</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="str">
+        <x:v>Preliminary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="8" t="str">
+        <x:v>wastewater_total_phosphorus</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="n">
+        <x:v>390481</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="str">
+        <x:v>tonnes</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E12" s="8" t="str">
+        <x:v>8-10 Main Pollutant Contents Discharged in Wastewater by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F12" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E08-10.jpg</x:v>
+      </x:c>
+      <x:c r="G12" s="8" t="str">
+        <x:v>Preliminary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="8" t="str">
+        <x:v>freight_total</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="n">
+        <x:v>5783625</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="str">
+        <x:v>10 000 tonnes</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="str">
+        <x:v>16-13 Freight Traffic by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F13" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-13.jpg</x:v>
+      </x:c>
+      <x:c r="G13" s="8" t="str">
+        <x:v>Includes 97072 not classified by region.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="8" t="str">
+        <x:v>enterprises</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="n">
+        <x:v>1605346</x:v>
+      </x:c>
+      <x:c r="C14" s="8" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D14" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E14" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F14" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G14" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="8" t="str">
+        <x:v>ecommerce_enterprises</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="n">
+        <x:v>205026</x:v>
+      </x:c>
+      <x:c r="C15" s="8" t="str">
+        <x:v>units</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E15" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F15" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G15" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>ecommerce_sales</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="n">
+        <x:v>386544</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>100 million yuan</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="E16" s="8" t="str">
+        <x:v>16-39 Informatization and E-Commerce of Enterprises by Region (2024)</x:v>
+      </x:c>
+      <x:c r="F16" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="G16" s="8" t="str">
+        <x:v>National printed value.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
@@ -11103,621 +14947,199 @@
         <x:v>The official statistical-system page explains that annual results are published through the yearbook.</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_02_05</x:v>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C19" s="8" t="str">
+        <x:v>Population at Year-end by Region</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>31 province-level regions, 2024</x:v>
+      </x:c>
+      <x:c r="E19" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E02-05.jpg</x:v>
+      </x:c>
+      <x:c r="F19" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G19" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H19" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I19" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J19" s="8" t="str">
+        <x:v>Social/demographic proxy only; the national total includes military personnel excluded from province rows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_06_18</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C20" s="8" t="str">
+        <x:v>Per Capita Disposable Income of Households by Region</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>31 province-level regions, 2024</x:v>
+      </x:c>
+      <x:c r="E20" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E06-18.jpg</x:v>
+      </x:c>
+      <x:c r="F20" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G20" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H20" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I20" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J20" s="8" t="str">
+        <x:v>Economic proxy; not a fishery-specific wage or coefficient series.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_08_10</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>Main Pollutant Contents Discharged in Wastewater by Region</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>31 province-level regions, 2024</x:v>
+      </x:c>
+      <x:c r="E21" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E08-10.jpg</x:v>
+      </x:c>
+      <x:c r="F21" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G21" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H21" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I21" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J21" s="8" t="str">
+        <x:v>Preliminary general wastewater data; not a fishery-water-quality measurement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_12_15</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>Output of Aquatic Products</x:v>
+      </x:c>
+      <x:c r="D22" s="8" t="str">
+        <x:v>31 province-level regions and national total, 2024</x:v>
+      </x:c>
+      <x:c r="E22" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E12-15.jpg</x:v>
+      </x:c>
+      <x:c r="F22" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G22" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H22" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I22" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J22" s="8" t="str">
+        <x:v>Primary public production backbone with marine/freshwater and capture/aquaculture components.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_16_13</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>Freight Traffic by Region</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>31 province-level regions, 2024</x:v>
+      </x:c>
+      <x:c r="E23" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-13.jpg</x:v>
+      </x:c>
+      <x:c r="F23" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G23" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H23" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I23" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J23" s="8" t="str">
+        <x:v>Economy-wide logistics proxy; national total contains a separately printed not-classified amount.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="8" t="str">
+        <x:v>nbs_yearbook_2025_table_16_39</x:v>
+      </x:c>
+      <x:c r="B24" s="8" t="str">
+        <x:v>National Bureau of Statistics of China</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="str">
+        <x:v>Informatization and E-Commerce of Enterprises by Region</x:v>
+      </x:c>
+      <x:c r="D24" s="8" t="str">
+        <x:v>31 province-level regions, 2024</x:v>
+      </x:c>
+      <x:c r="E24" s="8" t="str">
+        <x:v>https://www.stats.gov.cn/sj/ndsj/2025/html/E16-39.jpg</x:v>
+      </x:c>
+      <x:c r="F24" s="8" t="str">
+        <x:v>Official yearbook table downloaded and manually transcribed</x:v>
+      </x:c>
+      <x:c r="G24" s="8" t="str">
+        <x:v>Official website terms apply; numerical facts extracted with attribution</x:v>
+      </x:c>
+      <x:c r="H24" s="8" t="str">
+        <x:v>data/public/nbs_2024_31_province_public_panel.csv</x:v>
+      </x:c>
+      <x:c r="I24" s="8" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="J24" s="8" t="str">
+        <x:v>External digital/marketing proxy; not the paper's unreleased fishery EWM index.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="96" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="24" t="str">
-        <x:v>Public fishery data package</x:v>
-      </x:c>
-      <x:c r="B1" s="24" t="str">
-        <x:v>Review workbook for the GitHub reproduction repository</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="8" t="str">
-        <x:v>Retrieved</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
-        <x:v>2026-07-23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="8" t="str">
-        <x:v>Data label</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="str">
-        <x:v>经过处理的数据（公开来源） / processed data from public sources</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>World Bank / FAO</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Three China national production indicators, 2014-2023, CC BY 4.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="8" t="str">
-        <x:v>Ministry annual data</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="str">
-        <x:v>Accessible official HTML communiqués for 2015, 2016 and 2019-2024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="8" t="str">
-        <x:v>MOA 2024 detail</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>99 records: economy, species/water-body production, area, fleet, population, processing, trade and disasters</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="8" t="str">
-        <x:v>Fishery environment</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="str">
-        <x:v>12 records: monitoring network and reported exceedance-area change magnitudes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>Latest official</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="str">
-        <x:v>2025 national total/aquaculture/capture and Zhejiang total/marine/freshwater production</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="8" t="str">
-        <x:v>Reported vs normalized</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="str">
-        <x:v>Reported value/unit are retained; normalized value = reported value × normalization multiplier</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="8" t="str">
-        <x:v>Source integrity</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="str">
-        <x:v>Detailed rows contain the SHA-256 of the official HTML used by the parser</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="8" t="str">
-        <x:v>Province-level data</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>NBS indicator A0407 is documented, but its automated endpoint returned HTTP 403</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="28" t="str">
-        <x:v>Important</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="str">
-        <x:v>World Bank/FAO, Ministry and NBS totals can use different definitions; do not merge without checking scope</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="8" t="str">
-        <x:v>Missing values</x:v>
-      </x:c>
-      <x:c r="B13" s="8" t="str">
-        <x:v>not_found means the field was not located in that official HTML page; no interpolation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="8" t="str">
-        <x:v>Repository</x:v>
-      </x:c>
-      <x:c r="B14" s="8" t="str">
-        <x:v>https://github.com/niqundaye/Frontiers-in-Marine-Science</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="62" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="12" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="B1" s="12" t="str">
-        <x:v>Applies to</x:v>
-      </x:c>
-      <x:c r="C1" s="12" t="str">
-        <x:v>Meaning</x:v>
-      </x:c>
-      <x:c r="D1" s="12" t="str">
-        <x:v>Audit rule</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="8" t="str">
-        <x:v>year</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
-        <x:v>all data sheets</x:v>
-      </x:c>
-      <x:c r="C2" s="8" t="str">
-        <x:v>Reference year of the statistic</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="str">
-        <x:v>Integer year</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="8" t="str">
-        <x:v>section</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="str">
-        <x:v>MOA 2024 Detail</x:v>
-      </x:c>
-      <x:c r="C3" s="8" t="str">
-        <x:v>Communique topic group</x:v>
-      </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>Machine-readable text</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>indicator</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C4" s="8" t="str">
-        <x:v>Stable machine-readable indicator name</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="str">
-        <x:v>Do not translate in code</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="8" t="str">
-        <x:v>indicator_zh</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C5" s="8" t="str">
-        <x:v>Chinese label matching the official source concept</x:v>
-      </x:c>
-      <x:c r="D5" s="8" t="str">
-        <x:v>Human-readable</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="8" t="str">
-        <x:v>category</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>MOA 2024 Detail</x:v>
-      </x:c>
-      <x:c r="C6" s="8" t="str">
-        <x:v>Total/marine/freshwater or operational subgroup</x:v>
-      </x:c>
-      <x:c r="D6" s="8" t="str">
-        <x:v>Controls valid aggregation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="8" t="str">
-        <x:v>reported_value</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="str">
-        <x:v>Numeric value as displayed on the official page</x:v>
-      </x:c>
-      <x:c r="D7" s="8" t="str">
-        <x:v>Never overwrite</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>reported_unit</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="str">
-        <x:v>Unit as displayed on the official page</x:v>
-      </x:c>
-      <x:c r="D8" s="8" t="str">
-        <x:v>Never overwrite</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="8" t="str">
-        <x:v>normalization_multiplier</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C9" s="8" t="str">
-        <x:v>Exact multiplier used for unit conversion</x:v>
-      </x:c>
-      <x:c r="D9" s="8" t="str">
-        <x:v>value = reported_value × multiplier</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="8" t="str">
-        <x:v>value</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="str">
-        <x:v>all data sheets</x:v>
-      </x:c>
-      <x:c r="C10" s="8" t="str">
-        <x:v>Machine-readable normalized numeric value</x:v>
-      </x:c>
-      <x:c r="D10" s="8" t="str">
-        <x:v>Typed number</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="8" t="str">
-        <x:v>unit</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>all data sheets</x:v>
-      </x:c>
-      <x:c r="C11" s="8" t="str">
-        <x:v>Normalized unit</x:v>
-      </x:c>
-      <x:c r="D11" s="8" t="str">
-        <x:v>One unit per row</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="8" t="str">
-        <x:v>yoy_pct</x:v>
-      </x:c>
-      <x:c r="B12" s="8" t="str">
-        <x:v>MOA detail/latest</x:v>
-      </x:c>
-      <x:c r="C12" s="8" t="str">
-        <x:v>Signed year-on-year percent; declines are negative</x:v>
-      </x:c>
-      <x:c r="D12" s="8" t="str">
-        <x:v>Blank if source does not report</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="8" t="str">
-        <x:v>share_pct</x:v>
-      </x:c>
-      <x:c r="B13" s="8" t="str">
-        <x:v>MOA 2024 Detail</x:v>
-      </x:c>
-      <x:c r="C13" s="8" t="str">
-        <x:v>Share reported in source table</x:v>
-      </x:c>
-      <x:c r="D13" s="8" t="str">
-        <x:v>Blank unless explicitly reported</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="8" t="str">
-        <x:v>comparison_year</x:v>
-      </x:c>
-      <x:c r="B14" s="8" t="str">
-        <x:v>Environment 2024</x:v>
-      </x:c>
-      <x:c r="C14" s="8" t="str">
-        <x:v>Baseline year for a change indicator</x:v>
-      </x:c>
-      <x:c r="D14" s="8" t="str">
-        <x:v>Do not treat changes as levels</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="42" customHeight="1">
-      <x:c r="A15" s="8" t="str">
-        <x:v>change_direction</x:v>
-      </x:c>
-      <x:c r="B15" s="8" t="str">
-        <x:v>Environment 2024</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="str">
-        <x:v>level/increase/decrease classification</x:v>
-      </x:c>
-      <x:c r="D15" s="8" t="str">
-        <x:v>Interpret with comparison_year</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="42" customHeight="1">
-      <x:c r="A16" s="8" t="str">
-        <x:v>category_basis</x:v>
-      </x:c>
-      <x:c r="B16" s="8" t="str">
-        <x:v>Latest Official</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="str">
-        <x:v>Production method or water-body basis</x:v>
-      </x:c>
-      <x:c r="D16" s="8" t="str">
-        <x:v>Do not combine unlike bases</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="42" customHeight="1">
-      <x:c r="A17" s="8" t="str">
-        <x:v>source_url</x:v>
-      </x:c>
-      <x:c r="B17" s="8" t="str">
-        <x:v>all data sheets</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="str">
-        <x:v>Official page or API URL</x:v>
-      </x:c>
-      <x:c r="D17" s="8" t="str">
-        <x:v>Plain-text auditable URL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="42" customHeight="1">
-      <x:c r="A18" s="8" t="str">
-        <x:v>source_sha256</x:v>
-      </x:c>
-      <x:c r="B18" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="str">
-        <x:v>SHA-256 of downloaded official HTML</x:v>
-      </x:c>
-      <x:c r="D18" s="8" t="str">
-        <x:v>64 lowercase hexadecimal characters</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="42" customHeight="1">
-      <x:c r="A19" s="8" t="str">
-        <x:v>data_label</x:v>
-      </x:c>
-      <x:c r="B19" s="8" t="str">
-        <x:v>detailed/latest sheets</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="str">
-        <x:v>经过处理的数据（公开来源）</x:v>
-      </x:c>
-      <x:c r="D19" s="8" t="str">
-        <x:v>Never call author raw data</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="12" t="str">
-        <x:v>Check</x:v>
-      </x:c>
-      <x:c r="B1" s="12" t="str">
-        <x:v>Relationship</x:v>
-      </x:c>
-      <x:c r="C1" s="12" t="str">
-        <x:v>Difference</x:v>
-      </x:c>
-      <x:c r="D1" s="12" t="str">
-        <x:v>Tolerance</x:v>
-      </x:c>
-      <x:c r="E1" s="12" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="8" t="str">
-        <x:v>MOA detailed row count</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
-        <x:v>99 parsed records</x:v>
-      </x:c>
-      <x:c r="C2" s="20" t="n">
-        <x:f>COUNTA('MOA 2024 Detail'!A2:A100)-99</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D2" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E2" s="8" t="str">
-        <x:f>IF(ABS(C2)&lt;=D2,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="8" t="str">
-        <x:v>2024 economic output</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="str">
-        <x:v>total - fishery - industry/construction - circulation/services</x:v>
-      </x:c>
-      <x:c r="C3" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I61-'MOA 2024 Detail'!I55-'MOA 2024 Detail'!I54-'MOA 2024 Detail'!I53</x:f>
-        <x:v>1.8189894035458565e-12</x:v>
-      </x:c>
-      <x:c r="D3" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E3" s="8" t="str">
-        <x:f>IF(ABS(C3)&lt;=D3,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>2024 aquatic production</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>total - aquaculture - capture</x:v>
-      </x:c>
-      <x:c r="C4" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I100-'MOA 2024 Detail'!I94-'MOA 2024 Detail'!I96</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D4" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="str">
-        <x:f>IF(ABS(C4)&lt;=D4,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="8" t="str">
-        <x:v>2024 capture composition</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="str">
-        <x:v>capture - domestic capture - distant-water capture</x:v>
-      </x:c>
-      <x:c r="C5" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I96-'MOA 2024 Detail'!I35-'MOA 2024 Detail'!I97</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D5" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E5" s="8" t="str">
-        <x:f>IF(ABS(C5)&lt;=D5,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="8" t="str">
-        <x:v>2024 water-body composition</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>total - marine - freshwater</x:v>
-      </x:c>
-      <x:c r="C6" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I100-'MOA 2024 Detail'!I99-'MOA 2024 Detail'!I98</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E6" s="8" t="str">
-        <x:f>IF(ABS(C6)&lt;=D6,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="8" t="str">
-        <x:v>Motorized fleet tonnage</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="str">
-        <x:v>motorized - production - auxiliary (rounding allowed)</x:v>
-      </x:c>
-      <x:c r="C7" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I71-'MOA 2024 Detail'!I73-'MOA 2024 Detail'!I70</x:f>
-        <x:v>-100</x:v>
-      </x:c>
-      <x:c r="D7" s="20" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E7" s="8" t="str">
-        <x:f>IF(ABS(C7)&lt;=D7,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>Processed products</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="str">
-        <x:v>total - marine - freshwater (rounding allowed)</x:v>
-      </x:c>
-      <x:c r="C8" s="20" t="n">
-        <x:f>'MOA 2024 Detail'!I82-'MOA 2024 Detail'!I81-'MOA 2024 Detail'!I80</x:f>
-        <x:v>3.725290298461914e-9</x:v>
-      </x:c>
-      <x:c r="D8" s="20" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E8" s="8" t="str">
-        <x:f>IF(ABS(C8)&lt;=D8,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="8" t="str">
-        <x:v>2025 China production</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="str">
-        <x:v>total - aquaculture - capture</x:v>
-      </x:c>
-      <x:c r="C9" s="20" t="n">
-        <x:f>'Latest Official'!I2-'Latest Official'!I3-'Latest Official'!I4</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:f>IF(ABS(C9)&lt;=D9,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="8" t="str">
-        <x:v>2025 Zhejiang production</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="str">
-        <x:v>total - marine - freshwater</x:v>
-      </x:c>
-      <x:c r="C10" s="20" t="n">
-        <x:f>'Latest Official'!I5-'Latest Official'!I6-'Latest Official'!I7</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D10" s="20" t="n">
-        <x:v>0.000001</x:v>
-      </x:c>
-      <x:c r="E10" s="8" t="str">
-        <x:f>IF(ABS(C10)&lt;=D10,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E10">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="FAIL"/>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>